<commit_message>
Añadir hoja Puente P&L -> Caja al modelo de variaciones
Parte del EBITDA (enlazado del P&L Actual) y baja a caja con los deltas de
circulante del ST: Trade Receivables, Trade Payables & Accruals, Accruals l/p
y Deferred Income. Junio cuantificado y conciliado con la variacion de caja
real del balance. Replicable por mes pegando los saldos del ST.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRkTL6TNbSUmfpUN7nErPa
</commit_message>
<xml_diff>
--- a/Modelo_Variaciones_PL_2026.xlsx
+++ b/Modelo_Variaciones_PL_2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Variaciones" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Variaciones %" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Puente PL-Caja" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="#,##0;[Red](#,##0)"/>
     <numFmt numFmtId="165" formatCode="0.0%;[Red](0.0%)"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +75,12 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font/>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -135,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -176,6 +183,17 @@
     <xf numFmtId="165" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -850,19 +868,6 @@
           <t>BUDGET 2026 — P&amp;L mensual (€)</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="8" t="n"/>
-      <c r="G1" s="8" t="n"/>
-      <c r="H1" s="8" t="n"/>
-      <c r="I1" s="8" t="n"/>
-      <c r="J1" s="8" t="n"/>
-      <c r="K1" s="8" t="n"/>
-      <c r="L1" s="8" t="n"/>
-      <c r="M1" s="8" t="n"/>
-      <c r="N1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1776,19 +1781,6 @@
           <t>ACTUAL (ST) 2026 — P&amp;L mensual (€) · Junio cerrado</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="8" t="n"/>
-      <c r="G1" s="8" t="n"/>
-      <c r="H1" s="8" t="n"/>
-      <c r="I1" s="8" t="n"/>
-      <c r="J1" s="8" t="n"/>
-      <c r="K1" s="8" t="n"/>
-      <c r="L1" s="8" t="n"/>
-      <c r="M1" s="8" t="n"/>
-      <c r="N1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -2702,19 +2694,6 @@
           <t>VARIACIONES (Actual − Budget) €</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="8" t="n"/>
-      <c r="G1" s="8" t="n"/>
-      <c r="H1" s="8" t="n"/>
-      <c r="I1" s="8" t="n"/>
-      <c r="J1" s="8" t="n"/>
-      <c r="K1" s="8" t="n"/>
-      <c r="L1" s="8" t="n"/>
-      <c r="M1" s="8" t="n"/>
-      <c r="N1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -3772,19 +3751,6 @@
           <t>VARIACIONES % (vs Budget)</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="8" t="n"/>
-      <c r="G1" s="8" t="n"/>
-      <c r="H1" s="8" t="n"/>
-      <c r="I1" s="8" t="n"/>
-      <c r="J1" s="8" t="n"/>
-      <c r="K1" s="8" t="n"/>
-      <c r="L1" s="8" t="n"/>
-      <c r="M1" s="8" t="n"/>
-      <c r="N1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -4833,10 +4799,6 @@
           <t>DASHBOARD — Junio 2026 (Budget vs Actual)</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5102,4 +5064,783 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>PUENTE P&amp;L → CAJA (€k) — parte del EBITDA y baja a caja vía circulante</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+      <c r="F1" s="8" t="n"/>
+      <c r="G1" s="8" t="n"/>
+      <c r="H1" s="8" t="n"/>
+      <c r="I1" s="8" t="n"/>
+      <c r="J1" s="8" t="n"/>
+      <c r="K1" s="8" t="n"/>
+      <c r="L1" s="8" t="n"/>
+      <c r="M1" s="8" t="n"/>
+      <c r="N1" s="8" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Ene</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Abr</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>Ago</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>Dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>SALDOS DE BALANCE (€k)  ·  pega aquí del ST cada mes</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="11" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
+      <c r="N4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Trade &amp; Other Receivables (saldo)</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="12" t="n"/>
+      <c r="D5" s="12" t="n"/>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="12" t="n">
+        <v>62049</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>64297</v>
+      </c>
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="12" t="n"/>
+      <c r="L5" s="12" t="n"/>
+      <c r="M5" s="12" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Trade Payables &amp; Accruals c/p (saldo)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="12" t="n">
+        <v>278212</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>282393</v>
+      </c>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="12" t="n"/>
+      <c r="L6" s="12" t="n"/>
+      <c r="M6" s="12" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Accruals l/p (saldo)</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12" t="n">
+        <v>17873</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>17789</v>
+      </c>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="12" t="n"/>
+      <c r="M7" s="12" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Deferred Income - air traffic liab. (saldo)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n">
+        <v>195738</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>190268</v>
+      </c>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Equivalents (saldo)</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n">
+        <v>68882</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>54179</v>
+      </c>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="12" t="n"/>
+      <c r="M9" s="12" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>PUENTE P&amp;L → CAJA (€k)</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
+      <c r="N11" s="11" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>EBITDA (desde P&amp;L Actual)</t>
+        </is>
+      </c>
+      <c r="B12" s="12">
+        <f>'Actual (ST)'!B18/1000</f>
+        <v/>
+      </c>
+      <c r="C12" s="12">
+        <f>'Actual (ST)'!C18/1000</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>'Actual (ST)'!D18/1000</f>
+        <v/>
+      </c>
+      <c r="E12" s="12">
+        <f>'Actual (ST)'!E18/1000</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>'Actual (ST)'!F18/1000</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>'Actual (ST)'!G18/1000</f>
+        <v/>
+      </c>
+      <c r="H12" s="12">
+        <f>'Actual (ST)'!H18/1000</f>
+        <v/>
+      </c>
+      <c r="I12" s="12">
+        <f>'Actual (ST)'!I18/1000</f>
+        <v/>
+      </c>
+      <c r="J12" s="12">
+        <f>'Actual (ST)'!J18/1000</f>
+        <v/>
+      </c>
+      <c r="K12" s="12">
+        <f>'Actual (ST)'!K18/1000</f>
+        <v/>
+      </c>
+      <c r="L12" s="12">
+        <f>'Actual (ST)'!L18/1000</f>
+        <v/>
+      </c>
+      <c r="M12" s="12">
+        <f>'Actual (ST)'!M18/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>(−) Δ Trade Receivables</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="12">
+        <f>-(C5-B5)</f>
+        <v/>
+      </c>
+      <c r="D13" s="12">
+        <f>-(D5-C5)</f>
+        <v/>
+      </c>
+      <c r="E13" s="12">
+        <f>-(E5-D5)</f>
+        <v/>
+      </c>
+      <c r="F13" s="12">
+        <f>-(F5-E5)</f>
+        <v/>
+      </c>
+      <c r="G13" s="12">
+        <f>-(G5-F5)</f>
+        <v/>
+      </c>
+      <c r="H13" s="12">
+        <f>-(H5-G5)</f>
+        <v/>
+      </c>
+      <c r="I13" s="12">
+        <f>-(I5-H5)</f>
+        <v/>
+      </c>
+      <c r="J13" s="12">
+        <f>-(J5-I5)</f>
+        <v/>
+      </c>
+      <c r="K13" s="12">
+        <f>-(K5-J5)</f>
+        <v/>
+      </c>
+      <c r="L13" s="12">
+        <f>-(L5-K5)</f>
+        <v/>
+      </c>
+      <c r="M13" s="12">
+        <f>-(M5-L5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>(+) Δ Trade Payables &amp; Accruals</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="n"/>
+      <c r="C14" s="12">
+        <f>(C6-B6)</f>
+        <v/>
+      </c>
+      <c r="D14" s="12">
+        <f>(D6-C6)</f>
+        <v/>
+      </c>
+      <c r="E14" s="12">
+        <f>(E6-D6)</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>(F6-E6)</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>(G6-F6)</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>(H6-G6)</f>
+        <v/>
+      </c>
+      <c r="I14" s="12">
+        <f>(I6-H6)</f>
+        <v/>
+      </c>
+      <c r="J14" s="12">
+        <f>(J6-I6)</f>
+        <v/>
+      </c>
+      <c r="K14" s="12">
+        <f>(K6-J6)</f>
+        <v/>
+      </c>
+      <c r="L14" s="12">
+        <f>(L6-K6)</f>
+        <v/>
+      </c>
+      <c r="M14" s="12">
+        <f>(M6-L6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>(+) Δ Accruals l/p</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="n"/>
+      <c r="C15" s="12">
+        <f>(C7-B7)</f>
+        <v/>
+      </c>
+      <c r="D15" s="12">
+        <f>(D7-C7)</f>
+        <v/>
+      </c>
+      <c r="E15" s="12">
+        <f>(E7-D7)</f>
+        <v/>
+      </c>
+      <c r="F15" s="12">
+        <f>(F7-E7)</f>
+        <v/>
+      </c>
+      <c r="G15" s="12">
+        <f>(G7-F7)</f>
+        <v/>
+      </c>
+      <c r="H15" s="12">
+        <f>(H7-G7)</f>
+        <v/>
+      </c>
+      <c r="I15" s="12">
+        <f>(I7-H7)</f>
+        <v/>
+      </c>
+      <c r="J15" s="12">
+        <f>(J7-I7)</f>
+        <v/>
+      </c>
+      <c r="K15" s="12">
+        <f>(K7-J7)</f>
+        <v/>
+      </c>
+      <c r="L15" s="12">
+        <f>(L7-K7)</f>
+        <v/>
+      </c>
+      <c r="M15" s="12">
+        <f>(M7-L7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>(+) Δ Deferred Income</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="n"/>
+      <c r="C16" s="12">
+        <f>(C8-B8)</f>
+        <v/>
+      </c>
+      <c r="D16" s="12">
+        <f>(D8-C8)</f>
+        <v/>
+      </c>
+      <c r="E16" s="12">
+        <f>(E8-D8)</f>
+        <v/>
+      </c>
+      <c r="F16" s="12">
+        <f>(F8-E8)</f>
+        <v/>
+      </c>
+      <c r="G16" s="12">
+        <f>(G8-F8)</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>(H8-G8)</f>
+        <v/>
+      </c>
+      <c r="I16" s="12">
+        <f>(I8-H8)</f>
+        <v/>
+      </c>
+      <c r="J16" s="12">
+        <f>(J8-I8)</f>
+        <v/>
+      </c>
+      <c r="K16" s="12">
+        <f>(K8-J8)</f>
+        <v/>
+      </c>
+      <c r="L16" s="12">
+        <f>(L8-K8)</f>
+        <v/>
+      </c>
+      <c r="M16" s="12">
+        <f>(M8-L8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29">
+        <f> Variación Capital Circulante</f>
+        <v/>
+      </c>
+      <c r="B17" s="30" t="n"/>
+      <c r="C17" s="15">
+        <f>SUM(C13:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>SUM(D13:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>SUM(E13:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>SUM(F13:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="15">
+        <f>SUM(G13:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="15">
+        <f>SUM(H13:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="15">
+        <f>SUM(I13:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="15">
+        <f>SUM(J13:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="15">
+        <f>SUM(K13:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="15">
+        <f>SUM(L13:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="15">
+        <f>SUM(M13:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="29" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16">
+        <f> CASH FLOW OPERATIVO (EBITDA + circulante)</f>
+        <v/>
+      </c>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="17">
+        <f>C12+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="17">
+        <f>D12+D17</f>
+        <v/>
+      </c>
+      <c r="E18" s="17">
+        <f>E12+E17</f>
+        <v/>
+      </c>
+      <c r="F18" s="17">
+        <f>F12+F17</f>
+        <v/>
+      </c>
+      <c r="G18" s="17">
+        <f>G12+G17</f>
+        <v/>
+      </c>
+      <c r="H18" s="17">
+        <f>H12+H17</f>
+        <v/>
+      </c>
+      <c r="I18" s="17">
+        <f>I12+I17</f>
+        <v/>
+      </c>
+      <c r="J18" s="17">
+        <f>J12+J17</f>
+        <v/>
+      </c>
+      <c r="K18" s="17">
+        <f>K12+K17</f>
+        <v/>
+      </c>
+      <c r="L18" s="17">
+        <f>L12+L17</f>
+        <v/>
+      </c>
+      <c r="M18" s="17">
+        <f>M12+M17</f>
+        <v/>
+      </c>
+      <c r="N18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Δ Caja real (balance)</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="13">
+        <f>(C9-B9)</f>
+        <v/>
+      </c>
+      <c r="D19" s="13">
+        <f>(D9-C9)</f>
+        <v/>
+      </c>
+      <c r="E19" s="13">
+        <f>(E9-D9)</f>
+        <v/>
+      </c>
+      <c r="F19" s="13">
+        <f>(F9-E9)</f>
+        <v/>
+      </c>
+      <c r="G19" s="13">
+        <f>(G9-F9)</f>
+        <v/>
+      </c>
+      <c r="H19" s="13">
+        <f>(H9-G9)</f>
+        <v/>
+      </c>
+      <c r="I19" s="13">
+        <f>(I9-H9)</f>
+        <v/>
+      </c>
+      <c r="J19" s="13">
+        <f>(J9-I9)</f>
+        <v/>
+      </c>
+      <c r="K19" s="13">
+        <f>(K9-J9)</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>(L9-K9)</f>
+        <v/>
+      </c>
+      <c r="M19" s="13">
+        <f>(M9-L9)</f>
+        <v/>
+      </c>
+      <c r="N19" s="27" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>(=) Otros: financiación, leasing, capex, impuestos, intereses</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="n"/>
+      <c r="C20" s="34">
+        <f>C19-C18</f>
+        <v/>
+      </c>
+      <c r="D20" s="34">
+        <f>D19-D18</f>
+        <v/>
+      </c>
+      <c r="E20" s="34">
+        <f>E19-E18</f>
+        <v/>
+      </c>
+      <c r="F20" s="34">
+        <f>F19-F18</f>
+        <v/>
+      </c>
+      <c r="G20" s="34">
+        <f>G19-G18</f>
+        <v/>
+      </c>
+      <c r="H20" s="34">
+        <f>H19-H18</f>
+        <v/>
+      </c>
+      <c r="I20" s="34">
+        <f>I19-I18</f>
+        <v/>
+      </c>
+      <c r="J20" s="34">
+        <f>J19-J18</f>
+        <v/>
+      </c>
+      <c r="K20" s="34">
+        <f>K19-K18</f>
+        <v/>
+      </c>
+      <c r="L20" s="34">
+        <f>L19-L18</f>
+        <v/>
+      </c>
+      <c r="M20" s="34">
+        <f>M19-M18</f>
+        <v/>
+      </c>
+      <c r="N20" s="35" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="36" t="inlineStr">
+        <is>
+          <t>CÓMO USARLA: cada mes, pega los 5 saldos de balance del ST en la columna del mes (fila 5-9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t>El puente (fila 12-20) se recalcula solo: EBITDA + Δcirculante = Cash Flow Operativo; y concilia con la Δ de caja real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>Signos (efecto en CAJA): activo ↑ = caja ↓ (Receivables). Pasivo ↑ = caja ↑ (Payables, Accruals, Deferred Income).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>'Otros' = todo lo que hay bajo EBITDA y fuera de circulante (deuda, leasing IFRS16, capex, impuestos, intereses).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A26:N26"/>
+    <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A25:N25"/>
+    <mergeCell ref="A23:N23"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>